<commit_message>
Excel dynamic status update by finding status column
</commit_message>
<xml_diff>
--- a/vtiger-crm/src/test/resources/vtiger-excel-data.xlsx
+++ b/vtiger-crm/src/test/resources/vtiger-excel-data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="14295" windowHeight="6540" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="18030" windowHeight="6540" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Contact Data2" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="40">
   <si>
     <t>TC_ID</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Construction</t>
   </si>
   <si>
-    <t>Competitor</t>
-  </si>
-  <si>
     <t>PHNO</t>
   </si>
   <si>
@@ -138,20 +135,19 @@
     <t>Hello497</t>
   </si>
   <si>
-    <t>2026-04-28</t>
-  </si>
-  <si>
     <t>2026-05-31</t>
   </si>
   <si>
     <t>pass</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -763,7 +759,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -774,30 +770,30 @@
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.42578125"/>
-    <col min="2" max="2" customWidth="true" width="8.0"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="37.5703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="5" max="5" customWidth="true" width="13.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="22.7109375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="21.5703125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="1" max="1" width="7.42578125" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s" s="0">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -809,18 +805,18 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>28</v>
+      <c r="E2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>0</v>
@@ -829,12 +825,12 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F4" t="s" s="0">
+      <c r="F4" t="s">
         <v>3</v>
       </c>
     </row>
@@ -843,44 +839,44 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s" s="0">
-        <v>0</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E7" t="s" s="0">
+      <c r="E7" t="s">
         <v>2</v>
       </c>
-      <c r="F7" t="s" s="0">
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" t="s">
         <v>20</v>
       </c>
-      <c r="G7" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="H7" t="s" s="0">
+      <c r="H7" t="s">
         <v>3</v>
       </c>
     </row>
@@ -889,16 +885,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="F8" s="3">
         <v>46140</v>
@@ -906,8 +902,8 @@
       <c r="G8" s="3">
         <v>46143</v>
       </c>
-      <c r="H8" t="s" s="0">
-        <v>28</v>
+      <c r="H8" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -922,113 +918,102 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultColWidth="12.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" customWidth="true" width="29.85546875"/>
-    <col min="4" max="4" customWidth="true" width="15.5703125"/>
-    <col min="6" max="6" customWidth="true" style="4" width="21.85546875"/>
-    <col min="7" max="7" customWidth="true" style="4" width="20.28515625"/>
+    <col min="3" max="3" width="29.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s" s="0">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s" s="0">
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>17</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="4" t="s">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>33</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="0">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s" s="4">
-        <v>28</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="0">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s" s="0">
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="D3" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="F3" t="s" s="4">
-        <v>28</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="0">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s" s="0">
+      <c r="D4" t="s">
         <v>35</v>
       </c>
-      <c r="D4" t="s" s="0">
+      <c r="E4" t="s">
         <v>36</v>
       </c>
-      <c r="E4" t="s" s="0">
+      <c r="F4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="F6" s="4" t="s">
-        <v>28</v>
+      <c r="H4" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1042,127 +1027,127 @@
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="32.5703125"/>
+    <col min="3" max="3" width="32.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>13</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4">
+        <v>2783383839</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="I1" t="s" s="0">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="0">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="0">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>40</v>
-      </c>
-      <c r="I3" t="s" s="0">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="0">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s" s="0">
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="0">
-        <v>2783383839</v>
-      </c>
-      <c r="I4" t="s" s="0">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="0">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="H5" t="s" s="0">
-        <v>28</v>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:9">
-      <c r="F8" t="s" s="0">
-        <v>28</v>
+      <c r="F8" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
org data excel update
</commit_message>
<xml_diff>
--- a/vtiger-crm/src/test/resources/vtiger-excel-data.xlsx
+++ b/vtiger-crm/src/test/resources/vtiger-excel-data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="18030" windowHeight="6540" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="16320" windowHeight="6540" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Contact Data2" sheetId="2" r:id="rId1"/>
@@ -12,7 +12,7 @@
     <sheet name="Organization Data" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1:G20"/>
+  <oleSize ref="A1:M20"/>
   <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
     <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="40">
   <si>
     <t>TC_ID</t>
   </si>
@@ -138,10 +138,10 @@
     <t>2026-05-31</t>
   </si>
   <si>
-    <t>pass</t>
-  </si>
-  <si>
     <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>Analyst</t>
   </si>
 </sst>
 </file>
@@ -1007,7 +1007,7 @@
         <v>36</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>37</v>
@@ -1024,13 +1024,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1053,13 +1057,10 @@
         <v>12</v>
       </c>
       <c r="H1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1072,17 +1073,8 @@
       <c r="D2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1099,13 +1091,10 @@
         <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1119,13 +1108,10 @@
         <v>24</v>
       </c>
       <c r="G4">
-        <v>2783383839</v>
-      </c>
-      <c r="I4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>9348625285</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1137,17 +1123,6 @@
       </c>
       <c r="D5" t="s">
         <v>25</v>
-      </c>
-      <c r="G5" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="F8" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>